<commit_message>
Record weekly remaining hours in the sprint backlog
Fill in the amount of work remaining after each week of the sprint for
every task, ending with all tasks complete in week 4.
</commit_message>
<xml_diff>
--- a/documentation/Sprint_Backlog.xlsx
+++ b/documentation/Sprint_Backlog.xlsx
@@ -1456,10 +1456,18 @@
       <c r="C3" s="1">
         <v>0.5</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -1471,10 +1479,18 @@
       <c r="C4" s="1">
         <v>2</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="D4" s="2">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2">
+        <v>2</v>
+      </c>
+      <c r="F4" s="2">
+        <v>2</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1484,10 +1500,18 @@
       <c r="C5" s="1">
         <v>1</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -1499,10 +1523,18 @@
       <c r="C6" s="1">
         <v>2</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
+      <c r="D6" s="2">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2">
+        <v>2</v>
+      </c>
+      <c r="F6" s="2">
+        <v>2</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1512,10 +1544,18 @@
       <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="D7" s="2">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2">
+        <v>1</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
@@ -1525,10 +1565,18 @@
       <c r="C8" s="1">
         <v>0.5</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+      <c r="D8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -1540,10 +1588,18 @@
       <c r="C9" s="1">
         <v>1</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2">
+        <v>1</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
@@ -1553,10 +1609,18 @@
       <c r="C10" s="1">
         <v>1</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2">
+        <v>1</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -1568,10 +1632,18 @@
       <c r="C11" s="1">
         <v>0.5</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+      <c r="D11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
@@ -1581,10 +1653,18 @@
       <c r="C12" s="1">
         <v>0.5</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="D12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -1596,10 +1676,18 @@
       <c r="C13" s="1">
         <v>0.5</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="D13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
@@ -1609,10 +1697,18 @@
       <c r="C14" s="1">
         <v>0.5</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="D14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
@@ -1624,10 +1720,18 @@
       <c r="C15" s="1">
         <v>0.5</v>
       </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="D15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
@@ -1637,10 +1741,18 @@
       <c r="C16" s="1">
         <v>0.5</v>
       </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+      <c r="D16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
@@ -1652,10 +1764,18 @@
       <c r="C17" s="1">
         <v>2</v>
       </c>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+      <c r="D17" s="2">
+        <v>2</v>
+      </c>
+      <c r="E17" s="2">
+        <v>2</v>
+      </c>
+      <c r="F17" s="2">
+        <v>2</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
@@ -1665,10 +1785,18 @@
       <c r="C18" s="1">
         <v>1</v>
       </c>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="D18" s="2">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2">
+        <v>1</v>
+      </c>
+      <c r="F18" s="2">
+        <v>1</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
@@ -1680,10 +1808,18 @@
       <c r="C19" s="1">
         <v>1</v>
       </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+      <c r="D19" s="2">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2">
+        <v>1</v>
+      </c>
+      <c r="F19" s="2">
+        <v>1</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
@@ -1693,10 +1829,18 @@
       <c r="C20" s="1">
         <v>1</v>
       </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
+      <c r="D20" s="2">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2">
+        <v>1</v>
+      </c>
+      <c r="F20" s="2">
+        <v>1</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
@@ -1708,10 +1852,18 @@
       <c r="C21" s="1">
         <v>0.5</v>
       </c>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="D21" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E21" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F21" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G21" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
@@ -1721,10 +1873,18 @@
       <c r="C22" s="1">
         <v>0.5</v>
       </c>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="D22" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E22" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="F22" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="G22" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
@@ -1772,15 +1932,15 @@
       </c>
       <c r="D27" s="3">
         <f t="shared" ref="D27:G27" si="0">SUM(D3:D26)</f>
-        <v>0</v>
+        <v>17.5</v>
       </c>
       <c r="E27" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>17.5</v>
       </c>
       <c r="F27" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>17.5</v>
       </c>
       <c r="G27" s="3">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Record has been completed for search by vendor tasks in the sprint backlog
</commit_message>
<xml_diff>
--- a/documentation/Sprint_Backlog.xlsx
+++ b/documentation/Sprint_Backlog.xlsx
@@ -182,7 +182,7 @@
     <font>
       <sz val="18"/>
       <color indexed="8"/>
-      <name val="Calibri"/>
+      <name val="Helvetica Neue"/>
     </font>
     <font>
       <sz val="9"/>
@@ -195,7 +195,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -229,6 +229,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="14"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="15"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -331,7 +337,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -350,10 +356,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -365,31 +371,28 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="6" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="7" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -412,11 +415,11 @@
       <rgbColor rgb="ffa5a5a5"/>
       <rgbColor rgb="ffaaaaaa"/>
       <rgbColor rgb="ffbdd6ee"/>
+      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffececec"/>
       <rgbColor rgb="ffdeeaf6"/>
       <rgbColor rgb="ffb4c6e7"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffd8d8d8"/>
+      <rgbColor rgb="ffd9d9d9"/>
       <rgbColor rgb="ff595959"/>
     </indexedColors>
   </colors>
@@ -458,10 +461,10 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.378708"/>
+          <c:x val="0.378525"/>
           <c:y val="0"/>
-          <c:w val="0.242585"/>
-          <c:h val="0.125297"/>
+          <c:w val="0.242949"/>
+          <c:h val="0.126883"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -477,10 +480,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0685897"/>
-          <c:y val="0.125297"/>
-          <c:w val="0.92641"/>
-          <c:h val="0.799284"/>
+          <c:x val="0.0686927"/>
+          <c:y val="0.126883"/>
+          <c:w val="0.926307"/>
+          <c:h val="0.796902"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -505,7 +508,7 @@
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
-            <c:size val="4"/>
+            <c:size val="2"/>
             <c:spPr>
               <a:noFill/>
               <a:ln w="28575" cap="rnd">
@@ -519,7 +522,7 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
-            <c:numFmt formatCode="General" sourceLinked="1"/>
+            <c:numFmt formatCode="#,##0" sourceLinked="1"/>
             <c:txPr>
               <a:bodyPr/>
               <a:lstStyle/>
@@ -714,15 +717,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>357225</xdr:colOff>
+      <xdr:colOff>357224</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>91454</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>544195</xdr:colOff>
+      <xdr:colOff>536845</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>107170</xdr:rowOff>
+      <xdr:rowOff>76860</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -730,8 +733,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="11253825" y="607709"/>
-        <a:ext cx="4898670" cy="2424907"/>
+        <a:off x="11253824" y="607709"/>
+        <a:ext cx="4891322" cy="2394597"/>
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -937,17 +940,17 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -974,10 +977,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1216,12 +1219,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1498,7 +1501,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1525,10 +1528,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -2471,7 +2474,9 @@
       <c r="F23" s="13">
         <v>1</v>
       </c>
-      <c r="G23" s="16"/>
+      <c r="G23" s="14">
+        <v>0</v>
+      </c>
       <c r="H23" s="6"/>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
@@ -2499,7 +2504,9 @@
       <c r="F24" s="13">
         <v>1</v>
       </c>
-      <c r="G24" s="16"/>
+      <c r="G24" s="14">
+        <v>0</v>
+      </c>
       <c r="H24" s="6"/>
       <c r="I24" s="7"/>
       <c r="J24" s="7"/>
@@ -2527,7 +2534,9 @@
       <c r="F25" s="13">
         <v>1</v>
       </c>
-      <c r="G25" s="16"/>
+      <c r="G25" s="14">
+        <v>0</v>
+      </c>
       <c r="H25" s="6"/>
       <c r="I25" s="7"/>
       <c r="J25" s="7"/>
@@ -2555,7 +2564,9 @@
       <c r="F26" s="13">
         <v>0.5</v>
       </c>
-      <c r="G26" s="16"/>
+      <c r="G26" s="14">
+        <v>0</v>
+      </c>
       <c r="H26" s="6"/>
       <c r="I26" s="7"/>
       <c r="J26" s="7"/>
@@ -2567,27 +2578,27 @@
       <c r="P26" s="7"/>
     </row>
     <row r="27" ht="13.55" customHeight="1">
-      <c r="A27" s="17"/>
-      <c r="B27" t="s" s="18">
+      <c r="A27" s="16"/>
+      <c r="B27" t="s" s="17">
         <v>43</v>
       </c>
-      <c r="C27" s="19">
+      <c r="C27" s="18">
         <f>SUM(C3:C26)</f>
         <v>21.5</v>
       </c>
-      <c r="D27" s="19">
+      <c r="D27" s="18">
         <f>SUM(D3:D26)</f>
         <v>21</v>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="18">
         <f>SUM(E3:E26)</f>
         <v>21</v>
       </c>
-      <c r="F27" s="19">
+      <c r="F27" s="18">
         <f>SUM(F3:F26)</f>
         <v>21</v>
       </c>
-      <c r="G27" s="19">
+      <c r="G27" s="18">
         <f>SUM(G3:G26)</f>
         <v>0</v>
       </c>

</xml_diff>